<commit_message>
Kahoot: planilhas sem caracteres especiais (letras gregas e símbolos viram texto)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/quiz/kahoot/a09-kahoot.xlsx
+++ b/quiz/kahoot/a09-kahoot.xlsx
@@ -43,16 +43,16 @@
     <t>0 e 1</t>
   </si>
   <si>
-    <t>−∞ e +∞</t>
+    <t>-infinito e +infinito</t>
   </si>
   <si>
     <t>0 e 100</t>
   </si>
   <si>
-    <t>−1 e 1</t>
-  </si>
-  <si>
-    <t>Um r = −0,9 indica:</t>
+    <t>-1 e 1</t>
+  </si>
+  <si>
+    <t>Um r = -0,9 indica:</t>
   </si>
   <si>
     <t>Associação linear negativa fraca</t>
@@ -112,7 +112,7 @@
     <t>Filhos de pais muito altos tendem a ser menos altos que os pais</t>
   </si>
   <si>
-    <t>Em y = α + βx + ε, o que é β?</t>
+    <t>Em y = alfa + beta*x + erro, o que é beta?</t>
   </si>
   <si>
     <t>A correlação entre x e y</t>
@@ -142,7 +142,7 @@
     <t>Passa pelo maior número de pontos</t>
   </si>
   <si>
-    <t>Um R² = 0,64 significa que:</t>
+    <t>Um R2 = 0,64 significa que:</t>
   </si>
   <si>
     <t>64% dos pontos estão sobre a reta</t>
@@ -160,16 +160,16 @@
     <t>No teste da regressão, a hipótese nula é:</t>
   </si>
   <si>
-    <t>β = 0</t>
-  </si>
-  <si>
-    <t>α = 0</t>
-  </si>
-  <si>
-    <t>β ≠ 0</t>
-  </si>
-  <si>
-    <t>R² = 1</t>
+    <t>beta = 0</t>
+  </si>
+  <si>
+    <t>alfa = 0</t>
+  </si>
+  <si>
+    <t>beta diferente de 0</t>
+  </si>
+  <si>
+    <t>R2 = 1</t>
   </si>
   <si>
     <t>Resíduos em forma de funil indicam:</t>

</xml_diff>